<commit_message>
automate new period and building layout updates
- add missing periods automatically with preserved date formatting
- auto-detect and insert new building columns
- copy building and separator formatting from source workbook
- preserve worksheet layout when new buildings are added
</commit_message>
<xml_diff>
--- a/ref/testing_electricity_202604.xlsx
+++ b/ref/testing_electricity_202604.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tiffanychen/Desktop/intern/hkust_net_zero_office/sustainability-data-automation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tiffanychen/Desktop/intern/hkust_net_zero_office/sustainability-data-automation/ref/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{978A3109-FBD2-454A-81D2-CB9DD54988C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB0218FF-4736-564D-8BF8-41CE409C320E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3240" yWindow="780" windowWidth="26160" windowHeight="16780" tabRatio="887" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2560" yWindow="940" windowWidth="26160" windowHeight="16780" tabRatio="887" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CLP Tariff" sheetId="2" r:id="rId1"/>
@@ -350,7 +350,7 @@
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -359,12 +359,21 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-APCF Switches 1-33</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>APCF Switches 1-33</t>
         </r>
       </text>
     </comment>
@@ -422,7 +431,7 @@
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -431,12 +440,21 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Include cooling tower</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Include cooling tower</t>
         </r>
       </text>
     </comment>
@@ -3829,7 +3847,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="255">
   <si>
     <t>Total 
 (Group A) (kWh)</t>
@@ -4758,7 +4776,10 @@
     <t>RB2</t>
   </si>
   <si>
-    <t>HELLOOOO</t>
+    <t>TEST BUILDING 1</t>
+  </si>
+  <si>
+    <t>TEST BUILDING 2</t>
   </si>
 </sst>
 </file>
@@ -5294,7 +5315,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="79">
+  <fills count="80">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5747,6 +5768,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -6492,7 +6519,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="279">
+  <cellXfs count="280">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -7318,17 +7345,20 @@
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="49" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="49" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="79" borderId="34" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="110">
@@ -20494,10 +20524,9 @@
     <col min="29" max="29" width="2.5703125" style="4" customWidth="1"/>
     <col min="30" max="32" width="8.85546875" style="4"/>
     <col min="33" max="33" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="10.140625" style="4" customWidth="1"/>
-    <col min="36" max="36" width="9.5703125" style="4" customWidth="1"/>
-    <col min="37" max="37" width="10.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="9.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="10.140625" style="4" customWidth="1"/>
+    <col min="37" max="37" width="2.5703125" style="4" customWidth="1"/>
+    <col min="38" max="38" width="10.140625" style="4" customWidth="1"/>
     <col min="39" max="39" width="9.28515625" style="4" customWidth="1"/>
     <col min="40" max="40" width="10.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="9.28515625" style="4" customWidth="1"/>
@@ -20505,17 +20534,17 @@
     <col min="43" max="16384" width="8.85546875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" ht="29">
+    <row r="1" spans="1:38" ht="29">
       <c r="A1" s="15" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:36" ht="18.5" customHeight="1" thickBot="1">
+    <row r="2" spans="1:38" ht="18.5" customHeight="1" thickBot="1">
       <c r="A2" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:36" ht="65" thickBot="1">
+    <row r="3" spans="1:38" ht="65" thickBot="1">
       <c r="A3" s="222" t="s">
         <v>45</v>
       </c>
@@ -20618,11 +20647,14 @@
       <c r="AI3" s="251" t="s">
         <v>76</v>
       </c>
-      <c r="AJ3" s="4" t="s">
+      <c r="AJ3" s="279" t="s">
         <v>253</v>
       </c>
+      <c r="AL3" s="279" t="s">
+        <v>254</v>
+      </c>
     </row>
-    <row r="4" spans="1:36" ht="26" customHeight="1">
+    <row r="4" spans="1:38" ht="26" customHeight="1">
       <c r="A4" s="35">
         <v>41640</v>
       </c>
@@ -20721,8 +20753,10 @@
       </c>
       <c r="AH4" s="36"/>
       <c r="AI4" s="36"/>
+      <c r="AJ4" s="36"/>
+      <c r="AL4" s="36"/>
     </row>
-    <row r="5" spans="1:36" ht="23" customHeight="1">
+    <row r="5" spans="1:38" ht="23" customHeight="1">
       <c r="A5" s="35">
         <v>41671</v>
       </c>
@@ -20821,8 +20855,10 @@
       </c>
       <c r="AH5" s="37"/>
       <c r="AI5" s="37"/>
+      <c r="AJ5" s="37"/>
+      <c r="AL5" s="37"/>
     </row>
-    <row r="6" spans="1:36" ht="23" customHeight="1">
+    <row r="6" spans="1:38" ht="23" customHeight="1">
       <c r="A6" s="35">
         <v>41699</v>
       </c>
@@ -20921,8 +20957,10 @@
       </c>
       <c r="AH6" s="37"/>
       <c r="AI6" s="37"/>
+      <c r="AJ6" s="37"/>
+      <c r="AL6" s="37"/>
     </row>
-    <row r="7" spans="1:36" ht="22.25" customHeight="1">
+    <row r="7" spans="1:38" ht="22.25" customHeight="1">
       <c r="A7" s="35">
         <v>41730</v>
       </c>
@@ -21021,8 +21059,10 @@
       </c>
       <c r="AH7" s="37"/>
       <c r="AI7" s="37"/>
+      <c r="AJ7" s="37"/>
+      <c r="AL7" s="37"/>
     </row>
-    <row r="8" spans="1:36" ht="23.5" customHeight="1">
+    <row r="8" spans="1:38" ht="23.5" customHeight="1">
       <c r="A8" s="35">
         <v>41760</v>
       </c>
@@ -21121,8 +21161,10 @@
       </c>
       <c r="AH8" s="37"/>
       <c r="AI8" s="37"/>
+      <c r="AJ8" s="37"/>
+      <c r="AL8" s="37"/>
     </row>
-    <row r="9" spans="1:36" ht="25.25" customHeight="1">
+    <row r="9" spans="1:38" ht="25.25" customHeight="1">
       <c r="A9" s="35">
         <v>41791</v>
       </c>
@@ -21221,8 +21263,10 @@
       </c>
       <c r="AH9" s="37"/>
       <c r="AI9" s="37"/>
+      <c r="AJ9" s="37"/>
+      <c r="AL9" s="37"/>
     </row>
-    <row r="10" spans="1:36" ht="23.25" customHeight="1">
+    <row r="10" spans="1:38" ht="23.25" customHeight="1">
       <c r="A10" s="35">
         <v>41821</v>
       </c>
@@ -21321,8 +21365,10 @@
       </c>
       <c r="AH10" s="36"/>
       <c r="AI10" s="36"/>
+      <c r="AJ10" s="36"/>
+      <c r="AL10" s="36"/>
     </row>
-    <row r="11" spans="1:36" ht="23.25" customHeight="1">
+    <row r="11" spans="1:38" ht="23.25" customHeight="1">
       <c r="A11" s="39">
         <v>41852</v>
       </c>
@@ -21421,8 +21467,10 @@
       </c>
       <c r="AH11" s="40"/>
       <c r="AI11" s="40"/>
+      <c r="AJ11" s="40"/>
+      <c r="AL11" s="40"/>
     </row>
-    <row r="12" spans="1:36" ht="23.25" customHeight="1">
+    <row r="12" spans="1:38" ht="23.25" customHeight="1">
       <c r="A12" s="39">
         <v>41883</v>
       </c>
@@ -21521,8 +21569,10 @@
       </c>
       <c r="AH12" s="40"/>
       <c r="AI12" s="40"/>
+      <c r="AJ12" s="40"/>
+      <c r="AL12" s="40"/>
     </row>
-    <row r="13" spans="1:36" ht="23.25" customHeight="1">
+    <row r="13" spans="1:38" ht="23.25" customHeight="1">
       <c r="A13" s="39">
         <v>41913</v>
       </c>
@@ -21621,8 +21671,10 @@
       </c>
       <c r="AH13" s="40"/>
       <c r="AI13" s="40"/>
+      <c r="AJ13" s="40"/>
+      <c r="AL13" s="40"/>
     </row>
-    <row r="14" spans="1:36" ht="23.25" customHeight="1">
+    <row r="14" spans="1:38" ht="23.25" customHeight="1">
       <c r="A14" s="39">
         <v>41944</v>
       </c>
@@ -21721,8 +21773,10 @@
       </c>
       <c r="AH14" s="40"/>
       <c r="AI14" s="40"/>
+      <c r="AJ14" s="40"/>
+      <c r="AL14" s="40"/>
     </row>
-    <row r="15" spans="1:36" ht="23.25" customHeight="1">
+    <row r="15" spans="1:38" ht="23.25" customHeight="1">
       <c r="A15" s="39">
         <v>41974</v>
       </c>
@@ -21821,8 +21875,10 @@
       </c>
       <c r="AH15" s="40"/>
       <c r="AI15" s="40"/>
+      <c r="AJ15" s="40"/>
+      <c r="AL15" s="40"/>
     </row>
-    <row r="16" spans="1:36" ht="23.25" customHeight="1">
+    <row r="16" spans="1:38" ht="23.25" customHeight="1">
       <c r="A16" s="44">
         <v>42005</v>
       </c>
@@ -21921,8 +21977,10 @@
       </c>
       <c r="AH16" s="46"/>
       <c r="AI16" s="46"/>
+      <c r="AJ16" s="46"/>
+      <c r="AL16" s="46"/>
     </row>
-    <row r="17" spans="1:35" ht="23.25" customHeight="1">
+    <row r="17" spans="1:38" ht="23.25" customHeight="1">
       <c r="A17" s="44">
         <v>42036</v>
       </c>
@@ -22021,8 +22079,10 @@
       </c>
       <c r="AH17" s="46"/>
       <c r="AI17" s="46"/>
+      <c r="AJ17" s="46"/>
+      <c r="AL17" s="46"/>
     </row>
-    <row r="18" spans="1:35" ht="23.25" customHeight="1">
+    <row r="18" spans="1:38" ht="23.25" customHeight="1">
       <c r="A18" s="44">
         <v>42064</v>
       </c>
@@ -22121,8 +22181,10 @@
       </c>
       <c r="AH18" s="46"/>
       <c r="AI18" s="46"/>
+      <c r="AJ18" s="46"/>
+      <c r="AL18" s="46"/>
     </row>
-    <row r="19" spans="1:35" ht="23.25" customHeight="1">
+    <row r="19" spans="1:38" ht="23.25" customHeight="1">
       <c r="A19" s="44">
         <v>42095</v>
       </c>
@@ -22221,8 +22283,10 @@
       </c>
       <c r="AH19" s="45"/>
       <c r="AI19" s="45"/>
+      <c r="AJ19" s="45"/>
+      <c r="AL19" s="45"/>
     </row>
-    <row r="20" spans="1:35" ht="23.25" customHeight="1">
+    <row r="20" spans="1:38" ht="23.25" customHeight="1">
       <c r="A20" s="44">
         <v>42125</v>
       </c>
@@ -22321,8 +22385,10 @@
       </c>
       <c r="AH20" s="45"/>
       <c r="AI20" s="45"/>
+      <c r="AJ20" s="45"/>
+      <c r="AL20" s="45"/>
     </row>
-    <row r="21" spans="1:35" ht="23.25" customHeight="1">
+    <row r="21" spans="1:38" ht="23.25" customHeight="1">
       <c r="A21" s="44">
         <v>42156</v>
       </c>
@@ -22421,8 +22487,10 @@
       </c>
       <c r="AH21" s="45"/>
       <c r="AI21" s="45"/>
+      <c r="AJ21" s="45"/>
+      <c r="AL21" s="45"/>
     </row>
-    <row r="22" spans="1:35" ht="23.25" customHeight="1">
+    <row r="22" spans="1:38" ht="23.25" customHeight="1">
       <c r="A22" s="44">
         <v>42186</v>
       </c>
@@ -22521,8 +22589,10 @@
       </c>
       <c r="AH22" s="45"/>
       <c r="AI22" s="45"/>
+      <c r="AJ22" s="45"/>
+      <c r="AL22" s="45"/>
     </row>
-    <row r="23" spans="1:35" ht="23.25" customHeight="1">
+    <row r="23" spans="1:38" ht="23.25" customHeight="1">
       <c r="A23" s="44">
         <v>42217</v>
       </c>
@@ -22621,8 +22691,10 @@
       </c>
       <c r="AH23" s="45"/>
       <c r="AI23" s="45"/>
+      <c r="AJ23" s="45"/>
+      <c r="AL23" s="45"/>
     </row>
-    <row r="24" spans="1:35" ht="23.25" customHeight="1">
+    <row r="24" spans="1:38" ht="23.25" customHeight="1">
       <c r="A24" s="44">
         <v>42248</v>
       </c>
@@ -22721,8 +22793,10 @@
       </c>
       <c r="AH24" s="45"/>
       <c r="AI24" s="45"/>
+      <c r="AJ24" s="45"/>
+      <c r="AL24" s="45"/>
     </row>
-    <row r="25" spans="1:35" ht="23.25" customHeight="1">
+    <row r="25" spans="1:38" ht="23.25" customHeight="1">
       <c r="A25" s="44">
         <v>42278</v>
       </c>
@@ -22821,8 +22895,10 @@
       </c>
       <c r="AH25" s="45"/>
       <c r="AI25" s="45"/>
+      <c r="AJ25" s="45"/>
+      <c r="AL25" s="45"/>
     </row>
-    <row r="26" spans="1:35" ht="23.25" customHeight="1">
+    <row r="26" spans="1:38" ht="23.25" customHeight="1">
       <c r="A26" s="44">
         <v>42309</v>
       </c>
@@ -22921,8 +22997,10 @@
       </c>
       <c r="AH26" s="45"/>
       <c r="AI26" s="45"/>
+      <c r="AJ26" s="45"/>
+      <c r="AL26" s="45"/>
     </row>
-    <row r="27" spans="1:35" ht="23.25" customHeight="1">
+    <row r="27" spans="1:38" ht="23.25" customHeight="1">
       <c r="A27" s="44">
         <v>42339</v>
       </c>
@@ -23021,8 +23099,10 @@
       </c>
       <c r="AH27" s="45"/>
       <c r="AI27" s="45"/>
+      <c r="AJ27" s="45"/>
+      <c r="AL27" s="45"/>
     </row>
-    <row r="28" spans="1:35" ht="23.25" customHeight="1">
+    <row r="28" spans="1:38" ht="23.25" customHeight="1">
       <c r="A28" s="50">
         <v>42370</v>
       </c>
@@ -23121,8 +23201,10 @@
       </c>
       <c r="AH28" s="6"/>
       <c r="AI28" s="6"/>
+      <c r="AJ28" s="6"/>
+      <c r="AL28" s="6"/>
     </row>
-    <row r="29" spans="1:35" ht="23.25" customHeight="1">
+    <row r="29" spans="1:38" ht="23.25" customHeight="1">
       <c r="A29" s="50">
         <v>42401</v>
       </c>
@@ -23221,8 +23303,10 @@
       </c>
       <c r="AH29" s="6"/>
       <c r="AI29" s="6"/>
+      <c r="AJ29" s="6"/>
+      <c r="AL29" s="6"/>
     </row>
-    <row r="30" spans="1:35" ht="23.25" customHeight="1">
+    <row r="30" spans="1:38" ht="23.25" customHeight="1">
       <c r="A30" s="50">
         <v>42430</v>
       </c>
@@ -23321,8 +23405,10 @@
       </c>
       <c r="AH30" s="6"/>
       <c r="AI30" s="6"/>
+      <c r="AJ30" s="6"/>
+      <c r="AL30" s="6"/>
     </row>
-    <row r="31" spans="1:35" ht="23.25" customHeight="1">
+    <row r="31" spans="1:38" ht="23.25" customHeight="1">
       <c r="A31" s="50">
         <v>42461</v>
       </c>
@@ -23421,8 +23507,10 @@
       </c>
       <c r="AH31" s="6"/>
       <c r="AI31" s="6"/>
+      <c r="AJ31" s="6"/>
+      <c r="AL31" s="6"/>
     </row>
-    <row r="32" spans="1:35" ht="23.25" customHeight="1">
+    <row r="32" spans="1:38" ht="23.25" customHeight="1">
       <c r="A32" s="50">
         <v>42491</v>
       </c>
@@ -23521,8 +23609,10 @@
       </c>
       <c r="AH32" s="6"/>
       <c r="AI32" s="6"/>
+      <c r="AJ32" s="6"/>
+      <c r="AL32" s="6"/>
     </row>
-    <row r="33" spans="1:35" ht="23.25" customHeight="1">
+    <row r="33" spans="1:38" ht="23.25" customHeight="1">
       <c r="A33" s="50">
         <v>42522</v>
       </c>
@@ -23621,8 +23711,10 @@
       </c>
       <c r="AH33" s="6"/>
       <c r="AI33" s="6"/>
+      <c r="AJ33" s="6"/>
+      <c r="AL33" s="6"/>
     </row>
-    <row r="34" spans="1:35" ht="23.25" customHeight="1">
+    <row r="34" spans="1:38" ht="23.25" customHeight="1">
       <c r="A34" s="50">
         <v>42552</v>
       </c>
@@ -23721,8 +23813,10 @@
       </c>
       <c r="AH34" s="6"/>
       <c r="AI34" s="6"/>
+      <c r="AJ34" s="6"/>
+      <c r="AL34" s="6"/>
     </row>
-    <row r="35" spans="1:35" ht="23.25" customHeight="1">
+    <row r="35" spans="1:38" ht="23.25" customHeight="1">
       <c r="A35" s="50">
         <v>42583</v>
       </c>
@@ -23821,8 +23915,10 @@
       </c>
       <c r="AH35" s="12"/>
       <c r="AI35" s="12"/>
+      <c r="AJ35" s="12"/>
+      <c r="AL35" s="12"/>
     </row>
-    <row r="36" spans="1:35" ht="23.25" customHeight="1">
+    <row r="36" spans="1:38" ht="23.25" customHeight="1">
       <c r="A36" s="50">
         <v>42614</v>
       </c>
@@ -23921,8 +24017,10 @@
       </c>
       <c r="AH36" s="12"/>
       <c r="AI36" s="12"/>
+      <c r="AJ36" s="12"/>
+      <c r="AL36" s="12"/>
     </row>
-    <row r="37" spans="1:35" ht="23.25" customHeight="1">
+    <row r="37" spans="1:38" ht="23.25" customHeight="1">
       <c r="A37" s="50">
         <v>42644</v>
       </c>
@@ -24021,8 +24119,10 @@
       </c>
       <c r="AH37" s="12"/>
       <c r="AI37" s="12"/>
+      <c r="AJ37" s="12"/>
+      <c r="AL37" s="12"/>
     </row>
-    <row r="38" spans="1:35" ht="23.25" customHeight="1">
+    <row r="38" spans="1:38" ht="23.25" customHeight="1">
       <c r="A38" s="50">
         <v>42675</v>
       </c>
@@ -24121,8 +24221,10 @@
       </c>
       <c r="AH38" s="12"/>
       <c r="AI38" s="12"/>
+      <c r="AJ38" s="12"/>
+      <c r="AL38" s="12"/>
     </row>
-    <row r="39" spans="1:35" ht="23.25" customHeight="1">
+    <row r="39" spans="1:38" ht="23.25" customHeight="1">
       <c r="A39" s="50">
         <v>42705</v>
       </c>
@@ -24221,8 +24323,10 @@
       </c>
       <c r="AH39" s="12"/>
       <c r="AI39" s="12"/>
+      <c r="AJ39" s="12"/>
+      <c r="AL39" s="12"/>
     </row>
-    <row r="40" spans="1:35" ht="23.25" customHeight="1">
+    <row r="40" spans="1:38" ht="23.25" customHeight="1">
       <c r="A40" s="47">
         <v>42736</v>
       </c>
@@ -24321,8 +24425,10 @@
       </c>
       <c r="AH40" s="49"/>
       <c r="AI40" s="49"/>
+      <c r="AJ40" s="49"/>
+      <c r="AL40" s="49"/>
     </row>
-    <row r="41" spans="1:35" ht="23.25" customHeight="1">
+    <row r="41" spans="1:38" ht="23.25" customHeight="1">
       <c r="A41" s="47">
         <v>42767</v>
       </c>
@@ -24421,8 +24527,10 @@
       </c>
       <c r="AH41" s="49"/>
       <c r="AI41" s="49"/>
+      <c r="AJ41" s="49"/>
+      <c r="AL41" s="49"/>
     </row>
-    <row r="42" spans="1:35" ht="23.25" customHeight="1">
+    <row r="42" spans="1:38" ht="23.25" customHeight="1">
       <c r="A42" s="47">
         <v>42795</v>
       </c>
@@ -24521,8 +24629,10 @@
       </c>
       <c r="AH42" s="49"/>
       <c r="AI42" s="49"/>
+      <c r="AJ42" s="49"/>
+      <c r="AL42" s="49"/>
     </row>
-    <row r="43" spans="1:35" ht="23.25" customHeight="1">
+    <row r="43" spans="1:38" ht="23.25" customHeight="1">
       <c r="A43" s="47">
         <v>42826</v>
       </c>
@@ -24621,8 +24731,10 @@
       </c>
       <c r="AH43" s="48"/>
       <c r="AI43" s="48"/>
+      <c r="AJ43" s="48"/>
+      <c r="AL43" s="48"/>
     </row>
-    <row r="44" spans="1:35" ht="23.25" customHeight="1">
+    <row r="44" spans="1:38" ht="23.25" customHeight="1">
       <c r="A44" s="47">
         <v>42856</v>
       </c>
@@ -24721,8 +24833,10 @@
       </c>
       <c r="AH44" s="48"/>
       <c r="AI44" s="48"/>
+      <c r="AJ44" s="48"/>
+      <c r="AL44" s="48"/>
     </row>
-    <row r="45" spans="1:35" ht="23.25" customHeight="1">
+    <row r="45" spans="1:38" ht="23.25" customHeight="1">
       <c r="A45" s="47">
         <v>42887</v>
       </c>
@@ -24821,8 +24935,10 @@
       </c>
       <c r="AH45" s="48"/>
       <c r="AI45" s="48"/>
+      <c r="AJ45" s="48"/>
+      <c r="AL45" s="48"/>
     </row>
-    <row r="46" spans="1:35" ht="23.25" customHeight="1">
+    <row r="46" spans="1:38" ht="23.25" customHeight="1">
       <c r="A46" s="47">
         <v>42917</v>
       </c>
@@ -24921,8 +25037,10 @@
       </c>
       <c r="AH46" s="48"/>
       <c r="AI46" s="48"/>
+      <c r="AJ46" s="48"/>
+      <c r="AL46" s="48"/>
     </row>
-    <row r="47" spans="1:35" ht="23.25" customHeight="1">
+    <row r="47" spans="1:38" ht="23.25" customHeight="1">
       <c r="A47" s="47">
         <v>42948</v>
       </c>
@@ -25021,8 +25139,10 @@
       </c>
       <c r="AH47" s="48"/>
       <c r="AI47" s="48"/>
+      <c r="AJ47" s="48"/>
+      <c r="AL47" s="48"/>
     </row>
-    <row r="48" spans="1:35" ht="23.25" customHeight="1">
+    <row r="48" spans="1:38" ht="23.25" customHeight="1">
       <c r="A48" s="47">
         <v>42979</v>
       </c>
@@ -25121,8 +25241,10 @@
       </c>
       <c r="AH48" s="48"/>
       <c r="AI48" s="48"/>
+      <c r="AJ48" s="48"/>
+      <c r="AL48" s="48"/>
     </row>
-    <row r="49" spans="1:35" ht="23.25" customHeight="1">
+    <row r="49" spans="1:38" ht="23.25" customHeight="1">
       <c r="A49" s="47">
         <v>43009</v>
       </c>
@@ -25221,8 +25343,10 @@
       </c>
       <c r="AH49" s="48"/>
       <c r="AI49" s="48"/>
+      <c r="AJ49" s="48"/>
+      <c r="AL49" s="48"/>
     </row>
-    <row r="50" spans="1:35" ht="23.25" customHeight="1">
+    <row r="50" spans="1:38" ht="23.25" customHeight="1">
       <c r="A50" s="47">
         <v>43040</v>
       </c>
@@ -25321,8 +25445,10 @@
       </c>
       <c r="AH50" s="48"/>
       <c r="AI50" s="48"/>
+      <c r="AJ50" s="48"/>
+      <c r="AL50" s="48"/>
     </row>
-    <row r="51" spans="1:35" ht="23.25" customHeight="1">
+    <row r="51" spans="1:38" ht="23.25" customHeight="1">
       <c r="A51" s="47">
         <v>43070</v>
       </c>
@@ -25421,8 +25547,10 @@
       </c>
       <c r="AH51" s="48"/>
       <c r="AI51" s="48"/>
+      <c r="AJ51" s="48"/>
+      <c r="AL51" s="48"/>
     </row>
-    <row r="52" spans="1:35" ht="23.25" customHeight="1">
+    <row r="52" spans="1:38" ht="23.25" customHeight="1">
       <c r="A52" s="41">
         <v>43101</v>
       </c>
@@ -25521,8 +25649,10 @@
       </c>
       <c r="AH52" s="42"/>
       <c r="AI52" s="42"/>
+      <c r="AJ52" s="42"/>
+      <c r="AL52" s="42"/>
     </row>
-    <row r="53" spans="1:35" ht="23.25" customHeight="1">
+    <row r="53" spans="1:38" ht="23.25" customHeight="1">
       <c r="A53" s="41">
         <v>43132</v>
       </c>
@@ -25623,8 +25753,10 @@
       </c>
       <c r="AH53" s="42"/>
       <c r="AI53" s="42"/>
+      <c r="AJ53" s="42"/>
+      <c r="AL53" s="42"/>
     </row>
-    <row r="54" spans="1:35" ht="23.25" customHeight="1">
+    <row r="54" spans="1:38" ht="23.25" customHeight="1">
       <c r="A54" s="41">
         <v>43160</v>
       </c>
@@ -25725,8 +25857,10 @@
       </c>
       <c r="AH54" s="42"/>
       <c r="AI54" s="42"/>
+      <c r="AJ54" s="42"/>
+      <c r="AL54" s="42"/>
     </row>
-    <row r="55" spans="1:35" ht="23.25" customHeight="1">
+    <row r="55" spans="1:38" ht="23.25" customHeight="1">
       <c r="A55" s="41">
         <v>43191</v>
       </c>
@@ -25827,8 +25961,10 @@
       </c>
       <c r="AH55" s="42"/>
       <c r="AI55" s="42"/>
+      <c r="AJ55" s="42"/>
+      <c r="AL55" s="42"/>
     </row>
-    <row r="56" spans="1:35" ht="23.25" customHeight="1">
+    <row r="56" spans="1:38" ht="23.25" customHeight="1">
       <c r="A56" s="41">
         <v>43221</v>
       </c>
@@ -25929,8 +26065,10 @@
       </c>
       <c r="AH56" s="42"/>
       <c r="AI56" s="42"/>
+      <c r="AJ56" s="42"/>
+      <c r="AL56" s="42"/>
     </row>
-    <row r="57" spans="1:35" ht="23.25" customHeight="1">
+    <row r="57" spans="1:38" ht="23.25" customHeight="1">
       <c r="A57" s="41">
         <v>43252</v>
       </c>
@@ -26030,8 +26168,10 @@
       </c>
       <c r="AH57" s="43"/>
       <c r="AI57" s="43"/>
+      <c r="AJ57" s="43"/>
+      <c r="AL57" s="43"/>
     </row>
-    <row r="58" spans="1:35" ht="23.25" customHeight="1">
+    <row r="58" spans="1:38" ht="23.25" customHeight="1">
       <c r="A58" s="41">
         <v>43282</v>
       </c>
@@ -26131,8 +26271,10 @@
       </c>
       <c r="AH58" s="43"/>
       <c r="AI58" s="43"/>
+      <c r="AJ58" s="43"/>
+      <c r="AL58" s="43"/>
     </row>
-    <row r="59" spans="1:35" ht="23.25" customHeight="1">
+    <row r="59" spans="1:38" ht="23.25" customHeight="1">
       <c r="A59" s="41">
         <v>43313</v>
       </c>
@@ -26232,8 +26374,10 @@
       </c>
       <c r="AH59" s="43"/>
       <c r="AI59" s="43"/>
+      <c r="AJ59" s="43"/>
+      <c r="AL59" s="43"/>
     </row>
-    <row r="60" spans="1:35" ht="23.25" customHeight="1">
+    <row r="60" spans="1:38" ht="23.25" customHeight="1">
       <c r="A60" s="41">
         <v>43344</v>
       </c>
@@ -26333,8 +26477,10 @@
       </c>
       <c r="AH60" s="43"/>
       <c r="AI60" s="43"/>
+      <c r="AJ60" s="43"/>
+      <c r="AL60" s="43"/>
     </row>
-    <row r="61" spans="1:35" s="86" customFormat="1" ht="23.25" customHeight="1">
+    <row r="61" spans="1:38" s="86" customFormat="1" ht="23.25" customHeight="1">
       <c r="A61" s="102">
         <v>43374</v>
       </c>
@@ -26434,8 +26580,10 @@
       </c>
       <c r="AH61" s="43"/>
       <c r="AI61" s="43"/>
+      <c r="AJ61" s="43"/>
+      <c r="AL61" s="43"/>
     </row>
-    <row r="62" spans="1:35" ht="23.25" customHeight="1">
+    <row r="62" spans="1:38" ht="23.25" customHeight="1">
       <c r="A62" s="41">
         <v>43405</v>
       </c>
@@ -26535,8 +26683,10 @@
       </c>
       <c r="AH62" s="43"/>
       <c r="AI62" s="43"/>
+      <c r="AJ62" s="43"/>
+      <c r="AL62" s="43"/>
     </row>
-    <row r="63" spans="1:35" ht="23.25" customHeight="1">
+    <row r="63" spans="1:38" ht="23.25" customHeight="1">
       <c r="A63" s="41">
         <v>43435</v>
       </c>
@@ -26636,8 +26786,10 @@
       </c>
       <c r="AH63" s="43"/>
       <c r="AI63" s="43"/>
+      <c r="AJ63" s="43"/>
+      <c r="AL63" s="43"/>
     </row>
-    <row r="64" spans="1:35" ht="23.25" customHeight="1">
+    <row r="64" spans="1:38" ht="23.25" customHeight="1">
       <c r="A64" s="50">
         <v>43466</v>
       </c>
@@ -26737,8 +26889,10 @@
       </c>
       <c r="AH64" s="12"/>
       <c r="AI64" s="12"/>
+      <c r="AJ64" s="12"/>
+      <c r="AL64" s="12"/>
     </row>
-    <row r="65" spans="1:35" ht="23.25" customHeight="1">
+    <row r="65" spans="1:38" ht="23.25" customHeight="1">
       <c r="A65" s="50">
         <v>43497</v>
       </c>
@@ -26838,8 +26992,10 @@
       </c>
       <c r="AH65" s="12"/>
       <c r="AI65" s="12"/>
+      <c r="AJ65" s="12"/>
+      <c r="AL65" s="12"/>
     </row>
-    <row r="66" spans="1:35" ht="23.25" customHeight="1">
+    <row r="66" spans="1:38" ht="23.25" customHeight="1">
       <c r="A66" s="50">
         <v>43525</v>
       </c>
@@ -26939,8 +27095,10 @@
       </c>
       <c r="AH66" s="12"/>
       <c r="AI66" s="12"/>
+      <c r="AJ66" s="12"/>
+      <c r="AL66" s="12"/>
     </row>
-    <row r="67" spans="1:35" ht="23.25" customHeight="1">
+    <row r="67" spans="1:38" ht="23.25" customHeight="1">
       <c r="A67" s="50">
         <v>43556</v>
       </c>
@@ -27040,8 +27198,10 @@
       </c>
       <c r="AH67" s="6"/>
       <c r="AI67" s="6"/>
+      <c r="AJ67" s="6"/>
+      <c r="AL67" s="6"/>
     </row>
-    <row r="68" spans="1:35" ht="23.25" customHeight="1">
+    <row r="68" spans="1:38" ht="23.25" customHeight="1">
       <c r="A68" s="50">
         <v>43586</v>
       </c>
@@ -27141,8 +27301,10 @@
       </c>
       <c r="AH68" s="6"/>
       <c r="AI68" s="6"/>
+      <c r="AJ68" s="6"/>
+      <c r="AL68" s="6"/>
     </row>
-    <row r="69" spans="1:35" ht="23.25" customHeight="1">
+    <row r="69" spans="1:38" ht="23.25" customHeight="1">
       <c r="A69" s="50">
         <v>43617</v>
       </c>
@@ -27242,8 +27404,10 @@
       </c>
       <c r="AH69" s="6"/>
       <c r="AI69" s="6"/>
+      <c r="AJ69" s="6"/>
+      <c r="AL69" s="6"/>
     </row>
-    <row r="70" spans="1:35" ht="23.25" customHeight="1">
+    <row r="70" spans="1:38" ht="23.25" customHeight="1">
       <c r="A70" s="50">
         <v>43647</v>
       </c>
@@ -27343,8 +27507,10 @@
       </c>
       <c r="AH70" s="6"/>
       <c r="AI70" s="6"/>
+      <c r="AJ70" s="6"/>
+      <c r="AL70" s="6"/>
     </row>
-    <row r="71" spans="1:35" ht="23.25" customHeight="1">
+    <row r="71" spans="1:38" ht="23.25" customHeight="1">
       <c r="A71" s="50">
         <v>43678</v>
       </c>
@@ -27444,8 +27610,10 @@
       </c>
       <c r="AH71" s="6"/>
       <c r="AI71" s="6"/>
+      <c r="AJ71" s="6"/>
+      <c r="AL71" s="6"/>
     </row>
-    <row r="72" spans="1:35" ht="23.25" customHeight="1">
+    <row r="72" spans="1:38" ht="23.25" customHeight="1">
       <c r="A72" s="50">
         <v>43709</v>
       </c>
@@ -27545,8 +27713,10 @@
       </c>
       <c r="AH72" s="6"/>
       <c r="AI72" s="6"/>
+      <c r="AJ72" s="6"/>
+      <c r="AL72" s="6"/>
     </row>
-    <row r="73" spans="1:35" ht="23.25" customHeight="1">
+    <row r="73" spans="1:38" ht="23.25" customHeight="1">
       <c r="A73" s="50">
         <v>43739</v>
       </c>
@@ -27646,8 +27816,10 @@
       </c>
       <c r="AH73" s="12"/>
       <c r="AI73" s="12"/>
+      <c r="AJ73" s="12"/>
+      <c r="AL73" s="12"/>
     </row>
-    <row r="74" spans="1:35" ht="23.25" customHeight="1">
+    <row r="74" spans="1:38" ht="23.25" customHeight="1">
       <c r="A74" s="50">
         <v>43770</v>
       </c>
@@ -27747,8 +27919,10 @@
       </c>
       <c r="AH74" s="12"/>
       <c r="AI74" s="12"/>
+      <c r="AJ74" s="12"/>
+      <c r="AL74" s="12"/>
     </row>
-    <row r="75" spans="1:35" ht="23.25" customHeight="1">
+    <row r="75" spans="1:38" ht="23.25" customHeight="1">
       <c r="A75" s="50">
         <v>43800</v>
       </c>
@@ -27848,8 +28022,10 @@
       </c>
       <c r="AH75" s="12"/>
       <c r="AI75" s="12"/>
+      <c r="AJ75" s="12"/>
+      <c r="AL75" s="12"/>
     </row>
-    <row r="76" spans="1:35" ht="23.25" customHeight="1">
+    <row r="76" spans="1:38" ht="23.25" customHeight="1">
       <c r="A76" s="44">
         <v>43831</v>
       </c>
@@ -27949,8 +28125,10 @@
       </c>
       <c r="AH76" s="46"/>
       <c r="AI76" s="46"/>
+      <c r="AJ76" s="46"/>
+      <c r="AL76" s="46"/>
     </row>
-    <row r="77" spans="1:35" ht="23.25" customHeight="1">
+    <row r="77" spans="1:38" ht="23.25" customHeight="1">
       <c r="A77" s="44">
         <v>43862</v>
       </c>
@@ -28050,8 +28228,10 @@
       </c>
       <c r="AH77" s="46"/>
       <c r="AI77" s="46"/>
+      <c r="AJ77" s="46"/>
+      <c r="AL77" s="46"/>
     </row>
-    <row r="78" spans="1:35" ht="23.25" customHeight="1">
+    <row r="78" spans="1:38" ht="23.25" customHeight="1">
       <c r="A78" s="44">
         <v>43891</v>
       </c>
@@ -28151,8 +28331,10 @@
       </c>
       <c r="AH78" s="46"/>
       <c r="AI78" s="46"/>
+      <c r="AJ78" s="46"/>
+      <c r="AL78" s="46"/>
     </row>
-    <row r="79" spans="1:35" ht="23.25" customHeight="1">
+    <row r="79" spans="1:38" ht="23.25" customHeight="1">
       <c r="A79" s="44">
         <v>43922</v>
       </c>
@@ -28252,8 +28434,10 @@
       </c>
       <c r="AH79" s="46"/>
       <c r="AI79" s="46"/>
+      <c r="AJ79" s="46"/>
+      <c r="AL79" s="46"/>
     </row>
-    <row r="80" spans="1:35" ht="23.25" customHeight="1">
+    <row r="80" spans="1:38" ht="23.25" customHeight="1">
       <c r="A80" s="44">
         <v>43952</v>
       </c>
@@ -28353,8 +28537,10 @@
       </c>
       <c r="AH80" s="46"/>
       <c r="AI80" s="46"/>
+      <c r="AJ80" s="46"/>
+      <c r="AL80" s="46"/>
     </row>
-    <row r="81" spans="1:35" ht="23.25" customHeight="1">
+    <row r="81" spans="1:38" ht="23.25" customHeight="1">
       <c r="A81" s="44">
         <v>43983</v>
       </c>
@@ -28454,8 +28640,10 @@
       </c>
       <c r="AH81" s="46"/>
       <c r="AI81" s="46"/>
+      <c r="AJ81" s="46"/>
+      <c r="AL81" s="46"/>
     </row>
-    <row r="82" spans="1:35" ht="23.25" customHeight="1">
+    <row r="82" spans="1:38" ht="23.25" customHeight="1">
       <c r="A82" s="44">
         <v>44013</v>
       </c>
@@ -28555,8 +28743,10 @@
       </c>
       <c r="AH82" s="46"/>
       <c r="AI82" s="46"/>
+      <c r="AJ82" s="46"/>
+      <c r="AL82" s="46"/>
     </row>
-    <row r="83" spans="1:35" ht="23.25" customHeight="1">
+    <row r="83" spans="1:38" ht="23.25" customHeight="1">
       <c r="A83" s="44">
         <v>44044</v>
       </c>
@@ -28656,8 +28846,10 @@
       </c>
       <c r="AH83" s="46"/>
       <c r="AI83" s="46"/>
+      <c r="AJ83" s="46"/>
+      <c r="AL83" s="46"/>
     </row>
-    <row r="84" spans="1:35" ht="23.25" customHeight="1">
+    <row r="84" spans="1:38" ht="23.25" customHeight="1">
       <c r="A84" s="44">
         <v>44075</v>
       </c>
@@ -28757,8 +28949,10 @@
       </c>
       <c r="AH84" s="46"/>
       <c r="AI84" s="46"/>
+      <c r="AJ84" s="46"/>
+      <c r="AL84" s="46"/>
     </row>
-    <row r="85" spans="1:35" ht="23.25" customHeight="1">
+    <row r="85" spans="1:38" ht="23.25" customHeight="1">
       <c r="A85" s="44">
         <v>44105</v>
       </c>
@@ -28857,8 +29051,10 @@
       </c>
       <c r="AH85" s="46"/>
       <c r="AI85" s="46"/>
+      <c r="AJ85" s="46"/>
+      <c r="AL85" s="46"/>
     </row>
-    <row r="86" spans="1:35" ht="23.25" customHeight="1">
+    <row r="86" spans="1:38" ht="23.25" customHeight="1">
       <c r="A86" s="44">
         <v>44136</v>
       </c>
@@ -28957,8 +29153,10 @@
       </c>
       <c r="AH86" s="46"/>
       <c r="AI86" s="46"/>
+      <c r="AJ86" s="46"/>
+      <c r="AL86" s="46"/>
     </row>
-    <row r="87" spans="1:35" ht="23.25" customHeight="1">
+    <row r="87" spans="1:38" ht="23.25" customHeight="1">
       <c r="A87" s="44">
         <v>44166</v>
       </c>
@@ -29057,8 +29255,10 @@
       </c>
       <c r="AH87" s="46"/>
       <c r="AI87" s="46"/>
+      <c r="AJ87" s="46"/>
+      <c r="AL87" s="46"/>
     </row>
-    <row r="88" spans="1:35" ht="23.25" customHeight="1">
+    <row r="88" spans="1:38" ht="23.25" customHeight="1">
       <c r="A88" s="119">
         <v>44197</v>
       </c>
@@ -29157,8 +29357,10 @@
       </c>
       <c r="AH88" s="120"/>
       <c r="AI88" s="120"/>
+      <c r="AJ88" s="120"/>
+      <c r="AL88" s="120"/>
     </row>
-    <row r="89" spans="1:35" ht="23" customHeight="1">
+    <row r="89" spans="1:38" ht="23" customHeight="1">
       <c r="A89" s="119">
         <v>44228</v>
       </c>
@@ -29257,8 +29459,10 @@
       </c>
       <c r="AH89" s="120"/>
       <c r="AI89" s="120"/>
+      <c r="AJ89" s="120"/>
+      <c r="AL89" s="120"/>
     </row>
-    <row r="90" spans="1:35" ht="23.25" customHeight="1">
+    <row r="90" spans="1:38" ht="23.25" customHeight="1">
       <c r="A90" s="119">
         <v>44256</v>
       </c>
@@ -29357,8 +29561,10 @@
       </c>
       <c r="AH90" s="120"/>
       <c r="AI90" s="120"/>
+      <c r="AJ90" s="120"/>
+      <c r="AL90" s="120"/>
     </row>
-    <row r="91" spans="1:35" ht="23.25" customHeight="1">
+    <row r="91" spans="1:38" ht="23.25" customHeight="1">
       <c r="A91" s="119">
         <v>44287</v>
       </c>
@@ -29457,8 +29663,10 @@
       </c>
       <c r="AH91" s="120"/>
       <c r="AI91" s="120"/>
+      <c r="AJ91" s="120"/>
+      <c r="AL91" s="120"/>
     </row>
-    <row r="92" spans="1:35" ht="23.25" customHeight="1">
+    <row r="92" spans="1:38" ht="23.25" customHeight="1">
       <c r="A92" s="119">
         <v>44317</v>
       </c>
@@ -29557,8 +29765,10 @@
       </c>
       <c r="AH92" s="120"/>
       <c r="AI92" s="120"/>
+      <c r="AJ92" s="120"/>
+      <c r="AL92" s="120"/>
     </row>
-    <row r="93" spans="1:35" ht="23.25" customHeight="1">
+    <row r="93" spans="1:38" ht="23.25" customHeight="1">
       <c r="A93" s="119">
         <v>44348</v>
       </c>
@@ -29657,8 +29867,10 @@
       </c>
       <c r="AH93" s="120"/>
       <c r="AI93" s="120"/>
+      <c r="AJ93" s="120"/>
+      <c r="AL93" s="120"/>
     </row>
-    <row r="94" spans="1:35" ht="23.25" customHeight="1">
+    <row r="94" spans="1:38" ht="23.25" customHeight="1">
       <c r="A94" s="119">
         <v>44378</v>
       </c>
@@ -29757,8 +29969,10 @@
       </c>
       <c r="AH94" s="120"/>
       <c r="AI94" s="120"/>
+      <c r="AJ94" s="120"/>
+      <c r="AL94" s="120"/>
     </row>
-    <row r="95" spans="1:35" ht="23.25" customHeight="1">
+    <row r="95" spans="1:38" ht="23.25" customHeight="1">
       <c r="A95" s="119">
         <v>44409</v>
       </c>
@@ -29857,8 +30071,10 @@
       </c>
       <c r="AH95" s="120"/>
       <c r="AI95" s="120"/>
+      <c r="AJ95" s="120"/>
+      <c r="AL95" s="120"/>
     </row>
-    <row r="96" spans="1:35" ht="23.25" customHeight="1">
+    <row r="96" spans="1:38" ht="23.25" customHeight="1">
       <c r="A96" s="119">
         <v>44440</v>
       </c>
@@ -29957,8 +30173,10 @@
       </c>
       <c r="AH96" s="120"/>
       <c r="AI96" s="120"/>
+      <c r="AJ96" s="120"/>
+      <c r="AL96" s="120"/>
     </row>
-    <row r="97" spans="1:35" ht="23.25" customHeight="1">
+    <row r="97" spans="1:38" ht="23.25" customHeight="1">
       <c r="A97" s="119">
         <v>44470</v>
       </c>
@@ -30057,8 +30275,10 @@
       </c>
       <c r="AH97" s="120"/>
       <c r="AI97" s="120"/>
+      <c r="AJ97" s="120"/>
+      <c r="AL97" s="120"/>
     </row>
-    <row r="98" spans="1:35" ht="23.25" customHeight="1">
+    <row r="98" spans="1:38" ht="23.25" customHeight="1">
       <c r="A98" s="119">
         <v>44501</v>
       </c>
@@ -30157,8 +30377,10 @@
       </c>
       <c r="AH98" s="120"/>
       <c r="AI98" s="120"/>
+      <c r="AJ98" s="120"/>
+      <c r="AL98" s="120"/>
     </row>
-    <row r="99" spans="1:35" ht="23.25" customHeight="1">
+    <row r="99" spans="1:38" ht="23.25" customHeight="1">
       <c r="A99" s="119">
         <v>44531</v>
       </c>
@@ -30257,8 +30479,10 @@
       </c>
       <c r="AH99" s="120"/>
       <c r="AI99" s="120"/>
+      <c r="AJ99" s="120"/>
+      <c r="AL99" s="120"/>
     </row>
-    <row r="100" spans="1:35" ht="23.25" customHeight="1">
+    <row r="100" spans="1:38" ht="23.25" customHeight="1">
       <c r="A100" s="47">
         <v>44562</v>
       </c>
@@ -30354,8 +30578,10 @@
       </c>
       <c r="AH100" s="49"/>
       <c r="AI100" s="49"/>
+      <c r="AJ100" s="49"/>
+      <c r="AL100" s="49"/>
     </row>
-    <row r="101" spans="1:35" ht="23.25" customHeight="1">
+    <row r="101" spans="1:38" ht="23.25" customHeight="1">
       <c r="A101" s="47">
         <v>44593</v>
       </c>
@@ -30451,8 +30677,10 @@
       </c>
       <c r="AH101" s="49"/>
       <c r="AI101" s="49"/>
+      <c r="AJ101" s="49"/>
+      <c r="AL101" s="49"/>
     </row>
-    <row r="102" spans="1:35" ht="23.25" customHeight="1">
+    <row r="102" spans="1:38" ht="23.25" customHeight="1">
       <c r="A102" s="47">
         <v>44621</v>
       </c>
@@ -30551,8 +30779,10 @@
       </c>
       <c r="AH102" s="49"/>
       <c r="AI102" s="49"/>
+      <c r="AJ102" s="49"/>
+      <c r="AL102" s="49"/>
     </row>
-    <row r="103" spans="1:35" ht="23.25" customHeight="1">
+    <row r="103" spans="1:38" ht="23.25" customHeight="1">
       <c r="A103" s="47">
         <v>44652</v>
       </c>
@@ -30651,8 +30881,10 @@
       </c>
       <c r="AH103" s="49"/>
       <c r="AI103" s="49"/>
+      <c r="AJ103" s="49"/>
+      <c r="AL103" s="49"/>
     </row>
-    <row r="104" spans="1:35" ht="23.25" customHeight="1">
+    <row r="104" spans="1:38" ht="23.25" customHeight="1">
       <c r="A104" s="47">
         <v>44682</v>
       </c>
@@ -30751,8 +30983,10 @@
       </c>
       <c r="AH104" s="49"/>
       <c r="AI104" s="49"/>
+      <c r="AJ104" s="49"/>
+      <c r="AL104" s="49"/>
     </row>
-    <row r="105" spans="1:35" ht="23.25" customHeight="1">
+    <row r="105" spans="1:38" ht="23.25" customHeight="1">
       <c r="A105" s="47">
         <v>44713</v>
       </c>
@@ -30851,8 +31085,10 @@
       </c>
       <c r="AH105" s="49"/>
       <c r="AI105" s="49"/>
+      <c r="AJ105" s="49"/>
+      <c r="AL105" s="49"/>
     </row>
-    <row r="106" spans="1:35" ht="23.25" customHeight="1">
+    <row r="106" spans="1:38" ht="23.25" customHeight="1">
       <c r="A106" s="47">
         <v>44743</v>
       </c>
@@ -30951,8 +31187,10 @@
       </c>
       <c r="AH106" s="49"/>
       <c r="AI106" s="49"/>
+      <c r="AJ106" s="49"/>
+      <c r="AL106" s="49"/>
     </row>
-    <row r="107" spans="1:35" ht="23.25" customHeight="1">
+    <row r="107" spans="1:38" ht="23.25" customHeight="1">
       <c r="A107" s="47">
         <v>44774</v>
       </c>
@@ -31051,8 +31289,10 @@
       </c>
       <c r="AH107" s="49"/>
       <c r="AI107" s="49"/>
+      <c r="AJ107" s="49"/>
+      <c r="AL107" s="49"/>
     </row>
-    <row r="108" spans="1:35" ht="23.25" customHeight="1">
+    <row r="108" spans="1:38" ht="23.25" customHeight="1">
       <c r="A108" s="47">
         <v>44805</v>
       </c>
@@ -31151,8 +31391,10 @@
       </c>
       <c r="AH108" s="49"/>
       <c r="AI108" s="49"/>
+      <c r="AJ108" s="49"/>
+      <c r="AL108" s="49"/>
     </row>
-    <row r="109" spans="1:35" ht="23.25" customHeight="1">
+    <row r="109" spans="1:38" ht="23.25" customHeight="1">
       <c r="A109" s="47">
         <v>44835</v>
       </c>
@@ -31251,8 +31493,10 @@
       </c>
       <c r="AH109" s="49"/>
       <c r="AI109" s="49"/>
+      <c r="AJ109" s="49"/>
+      <c r="AL109" s="49"/>
     </row>
-    <row r="110" spans="1:35" ht="23.25" customHeight="1">
+    <row r="110" spans="1:38" ht="23.25" customHeight="1">
       <c r="A110" s="47">
         <v>44866</v>
       </c>
@@ -31351,8 +31595,10 @@
       </c>
       <c r="AH110" s="49"/>
       <c r="AI110" s="49"/>
+      <c r="AJ110" s="49"/>
+      <c r="AL110" s="49"/>
     </row>
-    <row r="111" spans="1:35" ht="23.25" customHeight="1">
+    <row r="111" spans="1:38" ht="23.25" customHeight="1">
       <c r="A111" s="47">
         <v>44896</v>
       </c>
@@ -31451,8 +31697,10 @@
       </c>
       <c r="AH111" s="49"/>
       <c r="AI111" s="49"/>
+      <c r="AJ111" s="49"/>
+      <c r="AL111" s="49"/>
     </row>
-    <row r="112" spans="1:35" ht="23.25" customHeight="1">
+    <row r="112" spans="1:38" ht="23.25" customHeight="1">
       <c r="A112" s="167">
         <v>44927</v>
       </c>
@@ -31553,8 +31801,10 @@
       </c>
       <c r="AH112" s="168"/>
       <c r="AI112" s="168"/>
+      <c r="AJ112" s="168"/>
+      <c r="AL112" s="168"/>
     </row>
-    <row r="113" spans="1:35" ht="23.25" customHeight="1">
+    <row r="113" spans="1:38" ht="23.25" customHeight="1">
       <c r="A113" s="167">
         <v>44958</v>
       </c>
@@ -31656,8 +31906,10 @@
       </c>
       <c r="AH113" s="168"/>
       <c r="AI113" s="168"/>
+      <c r="AJ113" s="168"/>
+      <c r="AL113" s="168"/>
     </row>
-    <row r="114" spans="1:35" ht="23.25" customHeight="1">
+    <row r="114" spans="1:38" ht="23.25" customHeight="1">
       <c r="A114" s="167">
         <v>44986</v>
       </c>
@@ -31757,8 +32009,10 @@
       </c>
       <c r="AH114" s="168"/>
       <c r="AI114" s="168"/>
+      <c r="AJ114" s="168"/>
+      <c r="AL114" s="168"/>
     </row>
-    <row r="115" spans="1:35" ht="23.25" customHeight="1">
+    <row r="115" spans="1:38" ht="23.25" customHeight="1">
       <c r="A115" s="167">
         <v>45017</v>
       </c>
@@ -31858,8 +32112,10 @@
       </c>
       <c r="AH115" s="168"/>
       <c r="AI115" s="168"/>
+      <c r="AJ115" s="168"/>
+      <c r="AL115" s="168"/>
     </row>
-    <row r="116" spans="1:35" ht="23.25" customHeight="1">
+    <row r="116" spans="1:38" ht="23.25" customHeight="1">
       <c r="A116" s="167">
         <v>45047</v>
       </c>
@@ -31959,8 +32215,10 @@
       </c>
       <c r="AH116" s="168"/>
       <c r="AI116" s="168"/>
+      <c r="AJ116" s="168"/>
+      <c r="AL116" s="168"/>
     </row>
-    <row r="117" spans="1:35" ht="23.25" customHeight="1">
+    <row r="117" spans="1:38" ht="23.25" customHeight="1">
       <c r="A117" s="167">
         <v>45078</v>
       </c>
@@ -32060,8 +32318,10 @@
       </c>
       <c r="AH117" s="168"/>
       <c r="AI117" s="168"/>
+      <c r="AJ117" s="168"/>
+      <c r="AL117" s="168"/>
     </row>
-    <row r="118" spans="1:35" ht="23.25" customHeight="1">
+    <row r="118" spans="1:38" ht="23.25" customHeight="1">
       <c r="A118" s="167">
         <v>45108</v>
       </c>
@@ -32161,8 +32421,10 @@
       </c>
       <c r="AH118" s="168"/>
       <c r="AI118" s="168"/>
+      <c r="AJ118" s="168"/>
+      <c r="AL118" s="168"/>
     </row>
-    <row r="119" spans="1:35" ht="23.25" customHeight="1">
+    <row r="119" spans="1:38" ht="23.25" customHeight="1">
       <c r="A119" s="167">
         <v>45139</v>
       </c>
@@ -32262,8 +32524,10 @@
       </c>
       <c r="AH119" s="168"/>
       <c r="AI119" s="168"/>
+      <c r="AJ119" s="168"/>
+      <c r="AL119" s="168"/>
     </row>
-    <row r="120" spans="1:35" ht="23.25" customHeight="1">
+    <row r="120" spans="1:38" ht="23.25" customHeight="1">
       <c r="A120" s="167">
         <v>45170</v>
       </c>
@@ -32363,8 +32627,10 @@
       </c>
       <c r="AH120" s="168"/>
       <c r="AI120" s="168"/>
+      <c r="AJ120" s="168"/>
+      <c r="AL120" s="168"/>
     </row>
-    <row r="121" spans="1:35" ht="23.25" customHeight="1">
+    <row r="121" spans="1:38" ht="23.25" customHeight="1">
       <c r="A121" s="167">
         <v>45200</v>
       </c>
@@ -32464,8 +32730,10 @@
       </c>
       <c r="AH121" s="168"/>
       <c r="AI121" s="168"/>
+      <c r="AJ121" s="168"/>
+      <c r="AL121" s="168"/>
     </row>
-    <row r="122" spans="1:35" ht="23.25" customHeight="1">
+    <row r="122" spans="1:38" ht="23.25" customHeight="1">
       <c r="A122" s="167">
         <v>45231</v>
       </c>
@@ -32565,8 +32833,10 @@
       </c>
       <c r="AH122" s="168"/>
       <c r="AI122" s="168"/>
+      <c r="AJ122" s="168"/>
+      <c r="AL122" s="168"/>
     </row>
-    <row r="123" spans="1:35" ht="23.25" customHeight="1">
+    <row r="123" spans="1:38" ht="23.25" customHeight="1">
       <c r="A123" s="167">
         <v>45261</v>
       </c>
@@ -32666,8 +32936,10 @@
       </c>
       <c r="AH123" s="168"/>
       <c r="AI123" s="168"/>
+      <c r="AJ123" s="168"/>
+      <c r="AL123" s="168"/>
     </row>
-    <row r="124" spans="1:35" ht="23.25" customHeight="1">
+    <row r="124" spans="1:38" ht="23.25" customHeight="1">
       <c r="A124" s="41">
         <v>45292</v>
       </c>
@@ -32767,8 +33039,10 @@
       </c>
       <c r="AH124" s="43"/>
       <c r="AI124" s="43"/>
+      <c r="AJ124" s="43"/>
+      <c r="AL124" s="43"/>
     </row>
-    <row r="125" spans="1:35" ht="23.25" customHeight="1">
+    <row r="125" spans="1:38" ht="23.25" customHeight="1">
       <c r="A125" s="41">
         <v>45323</v>
       </c>
@@ -32870,8 +33144,10 @@
       </c>
       <c r="AH125" s="43"/>
       <c r="AI125" s="43"/>
+      <c r="AJ125" s="43"/>
+      <c r="AL125" s="43"/>
     </row>
-    <row r="126" spans="1:35" ht="23.25" customHeight="1">
+    <row r="126" spans="1:38" ht="23.25" customHeight="1">
       <c r="A126" s="41">
         <v>45352</v>
       </c>
@@ -32973,8 +33249,10 @@
       </c>
       <c r="AH126" s="43"/>
       <c r="AI126" s="43"/>
+      <c r="AJ126" s="43"/>
+      <c r="AL126" s="43"/>
     </row>
-    <row r="127" spans="1:35" ht="23.25" customHeight="1">
+    <row r="127" spans="1:38" ht="23.25" customHeight="1">
       <c r="A127" s="41">
         <v>45383</v>
       </c>
@@ -33076,8 +33354,10 @@
       </c>
       <c r="AH127" s="43"/>
       <c r="AI127" s="43"/>
+      <c r="AJ127" s="43"/>
+      <c r="AL127" s="43"/>
     </row>
-    <row r="128" spans="1:35" ht="23.25" customHeight="1">
+    <row r="128" spans="1:38" ht="23.25" customHeight="1">
       <c r="A128" s="41">
         <v>45413</v>
       </c>
@@ -33181,6 +33461,8 @@
         <v>25801.31</v>
       </c>
       <c r="AI128" s="43"/>
+      <c r="AJ128" s="43"/>
+      <c r="AL128" s="43"/>
     </row>
     <row r="129" spans="1:38" ht="23.25" customHeight="1">
       <c r="A129" s="41">
@@ -33288,6 +33570,8 @@
       <c r="AI129" s="43">
         <v>317.89299999999997</v>
       </c>
+      <c r="AJ129" s="43"/>
+      <c r="AL129" s="43"/>
     </row>
     <row r="130" spans="1:38" ht="23.25" customHeight="1">
       <c r="A130" s="41">
@@ -33396,14 +33680,8 @@
       <c r="AI130" s="43">
         <v>7737.1329999999998</v>
       </c>
-      <c r="AK130" s="4">
-        <f>2311/3</f>
-        <v>770.33333333333337</v>
-      </c>
-      <c r="AL130" s="4">
-        <f>AK130*9</f>
-        <v>6933</v>
-      </c>
+      <c r="AJ130" s="43"/>
+      <c r="AL130" s="43"/>
     </row>
     <row r="131" spans="1:38" ht="23.25" customHeight="1">
       <c r="A131" s="41">
@@ -33511,6 +33789,8 @@
       <c r="AI131" s="43">
         <v>17199.11</v>
       </c>
+      <c r="AJ131" s="43"/>
+      <c r="AL131" s="43"/>
     </row>
     <row r="132" spans="1:38" ht="23.25" customHeight="1">
       <c r="A132" s="41">
@@ -33618,6 +33898,8 @@
       <c r="AI132" s="43">
         <v>13861.65</v>
       </c>
+      <c r="AJ132" s="43"/>
+      <c r="AL132" s="43"/>
     </row>
     <row r="133" spans="1:38" ht="23.25" customHeight="1">
       <c r="A133" s="41">
@@ -33723,6 +34005,8 @@
       <c r="AI133" s="43">
         <v>23632.76</v>
       </c>
+      <c r="AJ133" s="43"/>
+      <c r="AL133" s="43"/>
     </row>
     <row r="134" spans="1:38" ht="23.25" customHeight="1">
       <c r="A134" s="41">
@@ -33828,6 +34112,8 @@
       <c r="AI134" s="43">
         <v>23714.61</v>
       </c>
+      <c r="AJ134" s="43"/>
+      <c r="AL134" s="43"/>
     </row>
     <row r="135" spans="1:38" ht="23.25" customHeight="1">
       <c r="A135" s="41">
@@ -33934,6 +34220,8 @@
       <c r="AI135" s="43">
         <v>14599.27</v>
       </c>
+      <c r="AJ135" s="43"/>
+      <c r="AL135" s="43"/>
     </row>
     <row r="136" spans="1:38" ht="23.25" customHeight="1">
       <c r="A136" s="47">
@@ -34040,6 +34328,8 @@
       <c r="AI136" s="49">
         <v>24617.14</v>
       </c>
+      <c r="AJ136" s="49"/>
+      <c r="AL136" s="49"/>
     </row>
     <row r="137" spans="1:38" ht="23.25" customHeight="1">
       <c r="A137" s="47">
@@ -34148,6 +34438,8 @@
       <c r="AI137" s="49">
         <v>15191.66</v>
       </c>
+      <c r="AJ137" s="49"/>
+      <c r="AL137" s="49"/>
     </row>
     <row r="138" spans="1:38" ht="23.25" customHeight="1">
       <c r="A138" s="47">
@@ -34254,6 +34546,8 @@
       <c r="AI138" s="49">
         <v>23174.02</v>
       </c>
+      <c r="AJ138" s="49"/>
+      <c r="AL138" s="49"/>
     </row>
     <row r="139" spans="1:38" ht="23.25" customHeight="1">
       <c r="A139" s="47">
@@ -34362,6 +34656,8 @@
       <c r="AI139" s="49">
         <v>28426.29</v>
       </c>
+      <c r="AJ139" s="49"/>
+      <c r="AL139" s="49"/>
     </row>
     <row r="140" spans="1:38" ht="23.25" customHeight="1">
       <c r="A140" s="47">
@@ -34470,6 +34766,8 @@
       <c r="AI140" s="49">
         <v>32039</v>
       </c>
+      <c r="AJ140" s="49"/>
+      <c r="AL140" s="49"/>
     </row>
     <row r="141" spans="1:38" ht="23.25" customHeight="1">
       <c r="A141" s="47">
@@ -34577,6 +34875,8 @@
       <c r="AI141" s="49">
         <v>41319</v>
       </c>
+      <c r="AJ141" s="49"/>
+      <c r="AL141" s="49"/>
     </row>
     <row r="142" spans="1:38" ht="23.25" customHeight="1">
       <c r="A142" s="47">
@@ -34684,6 +34984,8 @@
       <c r="AI142" s="49">
         <v>41405</v>
       </c>
+      <c r="AJ142" s="49"/>
+      <c r="AL142" s="49"/>
     </row>
     <row r="143" spans="1:38" ht="23.25" customHeight="1">
       <c r="A143" s="47">
@@ -34795,6 +35097,8 @@
       <c r="AI143" s="49">
         <v>42556</v>
       </c>
+      <c r="AJ143" s="49"/>
+      <c r="AL143" s="49"/>
     </row>
     <row r="144" spans="1:38" ht="23.25" customHeight="1">
       <c r="A144" s="47">
@@ -34906,6 +35210,8 @@
       <c r="AI144" s="49">
         <v>36836</v>
       </c>
+      <c r="AJ144" s="49"/>
+      <c r="AL144" s="49"/>
     </row>
     <row r="145" spans="1:41" ht="23.25" customHeight="1">
       <c r="A145" s="47">
@@ -35016,6 +35322,8 @@
       <c r="AI145" s="49">
         <v>46903</v>
       </c>
+      <c r="AJ145" s="49"/>
+      <c r="AL145" s="49"/>
     </row>
     <row r="146" spans="1:41" ht="23.25" customHeight="1">
       <c r="A146" s="47">
@@ -35125,6 +35433,8 @@
       <c r="AI146" s="49">
         <v>47478</v>
       </c>
+      <c r="AJ146" s="49"/>
+      <c r="AL146" s="49"/>
     </row>
     <row r="147" spans="1:41" ht="23.25" customHeight="1">
       <c r="A147" s="47">
@@ -35234,6 +35544,8 @@
       <c r="AI147" s="49">
         <v>36034</v>
       </c>
+      <c r="AJ147" s="49"/>
+      <c r="AL147" s="49"/>
     </row>
     <row r="148" spans="1:41" ht="23.25" customHeight="1">
       <c r="A148" s="167">
@@ -35342,6 +35654,8 @@
       <c r="AI148" s="168">
         <v>48398</v>
       </c>
+      <c r="AJ148" s="168"/>
+      <c r="AL148" s="168"/>
     </row>
     <row r="149" spans="1:41" ht="23.25" customHeight="1">
       <c r="A149" s="167">
@@ -35450,9 +35764,10 @@
       <c r="AI149" s="168">
         <v>43012</v>
       </c>
-      <c r="AJ149" s="4">
-        <v>10000000</v>
-      </c>
+      <c r="AJ149" s="168">
+        <v>100000</v>
+      </c>
+      <c r="AL149" s="168"/>
     </row>
     <row r="150" spans="1:41" ht="23.25" customHeight="1">
       <c r="A150" s="167">
@@ -35561,6 +35876,10 @@
       <c r="AI150" s="168">
         <v>56770</v>
       </c>
+      <c r="AJ150" s="168"/>
+      <c r="AL150" s="168">
+        <v>200000000</v>
+      </c>
     </row>
     <row r="151" spans="1:41" ht="23.25" customHeight="1" thickBot="1">
       <c r="A151" s="167">
@@ -35670,6 +35989,8 @@
       <c r="AI151" s="168">
         <v>41971</v>
       </c>
+      <c r="AJ151" s="168"/>
+      <c r="AL151" s="168"/>
     </row>
     <row r="152" spans="1:41" ht="58.5" customHeight="1" thickBot="1">
       <c r="A152" s="222" t="s">
@@ -35774,7 +36095,8 @@
       <c r="AI152" s="231" t="s">
         <v>76</v>
       </c>
-      <c r="AK152"/>
+      <c r="AJ152" s="231"/>
+      <c r="AL152" s="231"/>
     </row>
     <row r="153" spans="1:41" ht="23.25" customHeight="1">
       <c r="A153" s="142" t="s">
@@ -35906,7 +36228,8 @@
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="AK153"/>
+      <c r="AJ153" s="123"/>
+      <c r="AL153" s="123"/>
     </row>
     <row r="154" spans="1:41" ht="23.25" customHeight="1">
       <c r="A154" s="142" t="s">
@@ -36044,7 +36367,8 @@
         <f>SUM(AI127:AI138)</f>
         <v>164045.24599999998</v>
       </c>
-      <c r="AK154"/>
+      <c r="AJ154" s="123"/>
+      <c r="AL154" s="123"/>
     </row>
     <row r="155" spans="1:41" s="144" customFormat="1" ht="23.25" customHeight="1">
       <c r="A155" s="142" t="s">
@@ -36183,8 +36507,9 @@
         <f>SUM(AI139:AI150)</f>
         <v>501176.29000000004</v>
       </c>
-      <c r="AJ155" s="4"/>
-      <c r="AK155"/>
+      <c r="AJ155" s="123"/>
+      <c r="AK155" s="4"/>
+      <c r="AL155" s="123"/>
     </row>
     <row r="156" spans="1:41" ht="23.25" customHeight="1">
       <c r="A156" s="142" t="s">
@@ -36302,7 +36627,8 @@
       <c r="AI156" s="143" t="s">
         <v>89</v>
       </c>
-      <c r="AK156"/>
+      <c r="AJ156" s="143"/>
+      <c r="AL156" s="143"/>
     </row>
     <row r="157" spans="1:41" ht="23.25" customHeight="1">
       <c r="A157" s="142" t="s">
@@ -36435,6 +36761,8 @@
         <f t="shared" si="53"/>
         <v>2.0551101127307283</v>
       </c>
+      <c r="AJ157" s="143"/>
+      <c r="AL157" s="143"/>
       <c r="AO157"/>
     </row>
     <row r="158" spans="1:41" ht="23.25" customHeight="1">
@@ -59035,7 +59363,7 @@
       </c>
     </row>
     <row r="47" spans="1:178">
-      <c r="A47" s="275"/>
+      <c r="A47" s="278"/>
       <c r="B47" s="265">
         <v>460823</v>
       </c>
@@ -59081,40 +59409,40 @@
       <c r="P47" s="274">
         <v>10325</v>
       </c>
-      <c r="Q47" s="277">
+      <c r="Q47" s="275">
         <v>12420</v>
       </c>
-      <c r="R47" s="277">
+      <c r="R47" s="275">
         <v>12770</v>
       </c>
-      <c r="S47" s="277">
+      <c r="S47" s="275">
         <v>17157</v>
       </c>
-      <c r="T47" s="277">
+      <c r="T47" s="275">
         <v>20679</v>
       </c>
-      <c r="U47" s="277">
+      <c r="U47" s="275">
         <v>21661</v>
       </c>
-      <c r="V47" s="277">
+      <c r="V47" s="275">
         <v>19687</v>
       </c>
-      <c r="W47" s="277">
+      <c r="W47" s="275">
         <v>19598</v>
       </c>
-      <c r="X47" s="277">
+      <c r="X47" s="275">
         <v>19579</v>
       </c>
-      <c r="Y47" s="277">
+      <c r="Y47" s="275">
         <v>23913</v>
       </c>
-      <c r="Z47" s="277">
+      <c r="Z47" s="275">
         <v>22106</v>
       </c>
-      <c r="AA47" s="277">
+      <c r="AA47" s="275">
         <v>20839</v>
       </c>
-      <c r="AB47" s="277">
+      <c r="AB47" s="275">
         <v>20632</v>
       </c>
       <c r="AC47" s="274">
@@ -59186,7 +59514,7 @@
       <c r="AY47" s="274">
         <v>19565</v>
       </c>
-      <c r="AZ47" s="278">
+      <c r="AZ47" s="277">
         <v>19146</v>
       </c>
       <c r="BA47" s="276">
@@ -59578,7 +59906,7 @@
       </c>
     </row>
     <row r="48" spans="1:178" customFormat="1" ht="17">
-      <c r="A48" s="275"/>
+      <c r="A48" s="278"/>
       <c r="B48" s="265">
         <v>205337</v>
       </c>
@@ -59600,18 +59928,18 @@
       <c r="N48" s="274"/>
       <c r="O48" s="274"/>
       <c r="P48" s="274"/>
-      <c r="Q48" s="277"/>
-      <c r="R48" s="277"/>
-      <c r="S48" s="277"/>
-      <c r="T48" s="277"/>
-      <c r="U48" s="277"/>
-      <c r="V48" s="277"/>
-      <c r="W48" s="277"/>
-      <c r="X48" s="277"/>
-      <c r="Y48" s="277"/>
-      <c r="Z48" s="277"/>
-      <c r="AA48" s="277"/>
-      <c r="AB48" s="277"/>
+      <c r="Q48" s="275"/>
+      <c r="R48" s="275"/>
+      <c r="S48" s="275"/>
+      <c r="T48" s="275"/>
+      <c r="U48" s="275"/>
+      <c r="V48" s="275"/>
+      <c r="W48" s="275"/>
+      <c r="X48" s="275"/>
+      <c r="Y48" s="275"/>
+      <c r="Z48" s="275"/>
+      <c r="AA48" s="275"/>
+      <c r="AB48" s="275"/>
       <c r="AC48" s="274"/>
       <c r="AD48" s="274"/>
       <c r="AE48" s="274"/>
@@ -59635,7 +59963,7 @@
       <c r="AW48" s="274"/>
       <c r="AX48" s="274"/>
       <c r="AY48" s="274"/>
-      <c r="AZ48" s="278"/>
+      <c r="AZ48" s="277"/>
       <c r="BA48" s="276"/>
       <c r="BB48" s="276"/>
       <c r="BC48" s="276"/>
@@ -60003,7 +60331,7 @@
       </c>
     </row>
     <row r="49" spans="1:178" customFormat="1" ht="34">
-      <c r="A49" s="275"/>
+      <c r="A49" s="278"/>
       <c r="B49" s="265">
         <v>229155</v>
       </c>
@@ -67790,50 +68118,6 @@
     </row>
   </sheetData>
   <mergeCells count="60">
-    <mergeCell ref="J47:J48"/>
-    <mergeCell ref="Q47:Q48"/>
-    <mergeCell ref="R47:R48"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="G47:G48"/>
-    <mergeCell ref="H47:H48"/>
-    <mergeCell ref="I47:I48"/>
-    <mergeCell ref="K47:K48"/>
-    <mergeCell ref="L47:L48"/>
-    <mergeCell ref="M47:M48"/>
-    <mergeCell ref="N47:N48"/>
-    <mergeCell ref="O47:O48"/>
-    <mergeCell ref="P47:P48"/>
-    <mergeCell ref="BJ47:BJ48"/>
-    <mergeCell ref="BD47:BD48"/>
-    <mergeCell ref="BE47:BE48"/>
-    <mergeCell ref="BF47:BF48"/>
-    <mergeCell ref="BG47:BG48"/>
-    <mergeCell ref="BH47:BH48"/>
-    <mergeCell ref="BI47:BI48"/>
-    <mergeCell ref="AP47:AP48"/>
-    <mergeCell ref="BC47:BC48"/>
-    <mergeCell ref="AR47:AR48"/>
-    <mergeCell ref="AS47:AS48"/>
-    <mergeCell ref="AT47:AT48"/>
-    <mergeCell ref="AU47:AU48"/>
-    <mergeCell ref="AV47:AV48"/>
-    <mergeCell ref="AW47:AW48"/>
-    <mergeCell ref="AX47:AX48"/>
-    <mergeCell ref="AY47:AY48"/>
-    <mergeCell ref="AZ47:AZ48"/>
-    <mergeCell ref="BA47:BA48"/>
-    <mergeCell ref="BB47:BB48"/>
-    <mergeCell ref="AK47:AK48"/>
-    <mergeCell ref="AL47:AL48"/>
-    <mergeCell ref="AM47:AM48"/>
-    <mergeCell ref="AN47:AN48"/>
-    <mergeCell ref="AO47:AO48"/>
-    <mergeCell ref="AF47:AF48"/>
-    <mergeCell ref="AG47:AG48"/>
-    <mergeCell ref="AH47:AH48"/>
-    <mergeCell ref="AI47:AI48"/>
-    <mergeCell ref="AJ47:AJ48"/>
     <mergeCell ref="AE47:AE48"/>
     <mergeCell ref="A47:A49"/>
     <mergeCell ref="BK47:BK48"/>
@@ -67850,6 +68134,50 @@
     <mergeCell ref="AC47:AC48"/>
     <mergeCell ref="AD47:AD48"/>
     <mergeCell ref="AQ47:AQ48"/>
+    <mergeCell ref="AF47:AF48"/>
+    <mergeCell ref="AG47:AG48"/>
+    <mergeCell ref="AH47:AH48"/>
+    <mergeCell ref="AI47:AI48"/>
+    <mergeCell ref="AJ47:AJ48"/>
+    <mergeCell ref="AK47:AK48"/>
+    <mergeCell ref="AL47:AL48"/>
+    <mergeCell ref="AM47:AM48"/>
+    <mergeCell ref="AN47:AN48"/>
+    <mergeCell ref="AO47:AO48"/>
+    <mergeCell ref="AP47:AP48"/>
+    <mergeCell ref="BC47:BC48"/>
+    <mergeCell ref="AR47:AR48"/>
+    <mergeCell ref="AS47:AS48"/>
+    <mergeCell ref="AT47:AT48"/>
+    <mergeCell ref="AU47:AU48"/>
+    <mergeCell ref="AV47:AV48"/>
+    <mergeCell ref="AW47:AW48"/>
+    <mergeCell ref="AX47:AX48"/>
+    <mergeCell ref="AY47:AY48"/>
+    <mergeCell ref="AZ47:AZ48"/>
+    <mergeCell ref="BA47:BA48"/>
+    <mergeCell ref="BB47:BB48"/>
+    <mergeCell ref="BJ47:BJ48"/>
+    <mergeCell ref="BD47:BD48"/>
+    <mergeCell ref="BE47:BE48"/>
+    <mergeCell ref="BF47:BF48"/>
+    <mergeCell ref="BG47:BG48"/>
+    <mergeCell ref="BH47:BH48"/>
+    <mergeCell ref="BI47:BI48"/>
+    <mergeCell ref="J47:J48"/>
+    <mergeCell ref="Q47:Q48"/>
+    <mergeCell ref="R47:R48"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="G47:G48"/>
+    <mergeCell ref="H47:H48"/>
+    <mergeCell ref="I47:I48"/>
+    <mergeCell ref="K47:K48"/>
+    <mergeCell ref="L47:L48"/>
+    <mergeCell ref="M47:M48"/>
+    <mergeCell ref="N47:N48"/>
+    <mergeCell ref="O47:O48"/>
+    <mergeCell ref="P47:P48"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
@@ -68138,15 +68466,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Loretta xmlns="bc76fe4c-a155-4cd4-b3ce-e749a30fe160" xsi:nil="true"/>
@@ -68159,6 +68478,15 @@
     <TaxCatchAll xmlns="be3055c3-5ee9-432b-9d2b-e9bb13d3524a" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -68181,14 +68509,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4277783-1FC0-4518-9AC7-78441643C7FE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{771927D8-23AB-4166-821E-2FB8CF69E88F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -68197,4 +68517,12 @@
     <ds:schemaRef ds:uri="be3055c3-5ee9-432b-9d2b-e9bb13d3524a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4277783-1FC0-4518-9AC7-78441643C7FE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fixed color issues + optimized design
</commit_message>
<xml_diff>
--- a/ref/testing_electricity_202604.xlsx
+++ b/ref/testing_electricity_202604.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tiffanychen/Desktop/intern/hkust_net_zero_office/sustainability-data-automation/ref/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB0218FF-4736-564D-8BF8-41CE409C320E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6765342E-D962-934C-8A95-42D661D79C68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2560" yWindow="940" windowWidth="26160" windowHeight="16780" tabRatio="887" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2560" yWindow="820" windowWidth="26160" windowHeight="16780" tabRatio="887" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CLP Tariff" sheetId="2" r:id="rId1"/>
@@ -7336,6 +7336,9 @@
     <xf numFmtId="0" fontId="42" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="79" borderId="34" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="76" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -7356,9 +7359,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="79" borderId="34" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="110">
@@ -13093,13 +13093,13 @@
       <c r="D1" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="272" t="s">
+      <c r="E1" s="273" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="273"/>
-      <c r="G1" s="273"/>
-      <c r="H1" s="273"/>
-      <c r="I1" s="273"/>
+      <c r="F1" s="274"/>
+      <c r="G1" s="274"/>
+      <c r="H1" s="274"/>
+      <c r="I1" s="274"/>
       <c r="J1" s="185"/>
       <c r="K1" s="253" t="s">
         <v>4</v>
@@ -20647,10 +20647,10 @@
       <c r="AI3" s="251" t="s">
         <v>76</v>
       </c>
-      <c r="AJ3" s="279" t="s">
+      <c r="AJ3" s="272" t="s">
         <v>253</v>
       </c>
-      <c r="AL3" s="279" t="s">
+      <c r="AL3" s="272" t="s">
         <v>254</v>
       </c>
     </row>
@@ -35767,7 +35767,9 @@
       <c r="AJ149" s="168">
         <v>100000</v>
       </c>
-      <c r="AL149" s="168"/>
+      <c r="AL149" s="168">
+        <v>200000000</v>
+      </c>
     </row>
     <row r="150" spans="1:41" ht="23.25" customHeight="1">
       <c r="A150" s="167">
@@ -35876,7 +35878,9 @@
       <c r="AI150" s="168">
         <v>56770</v>
       </c>
-      <c r="AJ150" s="168"/>
+      <c r="AJ150" s="168">
+        <v>100000</v>
+      </c>
       <c r="AL150" s="168">
         <v>200000000</v>
       </c>
@@ -35989,8 +35993,12 @@
       <c r="AI151" s="168">
         <v>41971</v>
       </c>
-      <c r="AJ151" s="168"/>
-      <c r="AL151" s="168"/>
+      <c r="AJ151" s="168">
+        <v>100000</v>
+      </c>
+      <c r="AL151" s="168">
+        <v>200000000</v>
+      </c>
     </row>
     <row r="152" spans="1:41" ht="58.5" customHeight="1" thickBot="1">
       <c r="A152" s="222" t="s">
@@ -59363,7 +59371,7 @@
       </c>
     </row>
     <row r="47" spans="1:178">
-      <c r="A47" s="278"/>
+      <c r="A47" s="279"/>
       <c r="B47" s="265">
         <v>460823</v>
       </c>
@@ -59373,181 +59381,181 @@
       <c r="D47" s="163" t="s">
         <v>232</v>
       </c>
-      <c r="E47" s="274">
-        <v>0</v>
-      </c>
-      <c r="F47" s="274">
+      <c r="E47" s="275">
+        <v>0</v>
+      </c>
+      <c r="F47" s="275">
         <v>5475</v>
       </c>
-      <c r="G47" s="274">
+      <c r="G47" s="275">
         <v>16458</v>
       </c>
-      <c r="H47" s="274">
+      <c r="H47" s="275">
         <v>17218</v>
       </c>
-      <c r="I47" s="274">
+      <c r="I47" s="275">
         <v>17679</v>
       </c>
-      <c r="J47" s="274">
+      <c r="J47" s="275">
         <v>13495</v>
       </c>
-      <c r="K47" s="274">
+      <c r="K47" s="275">
         <v>13403</v>
       </c>
-      <c r="L47" s="274">
+      <c r="L47" s="275">
         <v>12981</v>
       </c>
-      <c r="M47" s="274">
+      <c r="M47" s="275">
         <v>14555</v>
       </c>
-      <c r="N47" s="274">
+      <c r="N47" s="275">
         <v>15328</v>
       </c>
-      <c r="O47" s="274">
+      <c r="O47" s="275">
         <v>14210</v>
       </c>
-      <c r="P47" s="274">
+      <c r="P47" s="275">
         <v>10325</v>
       </c>
-      <c r="Q47" s="275">
+      <c r="Q47" s="276">
         <v>12420</v>
       </c>
-      <c r="R47" s="275">
+      <c r="R47" s="276">
         <v>12770</v>
       </c>
-      <c r="S47" s="275">
+      <c r="S47" s="276">
         <v>17157</v>
       </c>
-      <c r="T47" s="275">
+      <c r="T47" s="276">
         <v>20679</v>
       </c>
-      <c r="U47" s="275">
+      <c r="U47" s="276">
         <v>21661</v>
       </c>
-      <c r="V47" s="275">
+      <c r="V47" s="276">
         <v>19687</v>
       </c>
-      <c r="W47" s="275">
+      <c r="W47" s="276">
         <v>19598</v>
       </c>
-      <c r="X47" s="275">
+      <c r="X47" s="276">
         <v>19579</v>
       </c>
-      <c r="Y47" s="275">
+      <c r="Y47" s="276">
         <v>23913</v>
       </c>
-      <c r="Z47" s="275">
+      <c r="Z47" s="276">
         <v>22106</v>
       </c>
-      <c r="AA47" s="275">
+      <c r="AA47" s="276">
         <v>20839</v>
       </c>
-      <c r="AB47" s="275">
+      <c r="AB47" s="276">
         <v>20632</v>
       </c>
-      <c r="AC47" s="274">
+      <c r="AC47" s="275">
         <v>18836</v>
       </c>
-      <c r="AD47" s="274">
+      <c r="AD47" s="275">
         <v>19648</v>
       </c>
-      <c r="AE47" s="274">
+      <c r="AE47" s="275">
         <v>26799</v>
       </c>
-      <c r="AF47" s="274">
+      <c r="AF47" s="275">
         <v>25388</v>
       </c>
-      <c r="AG47" s="274">
+      <c r="AG47" s="275">
         <v>25624</v>
       </c>
-      <c r="AH47" s="274">
+      <c r="AH47" s="275">
         <v>20185</v>
       </c>
-      <c r="AI47" s="274">
+      <c r="AI47" s="275">
         <v>19159</v>
       </c>
-      <c r="AJ47" s="274">
+      <c r="AJ47" s="275">
         <v>21519</v>
       </c>
-      <c r="AK47" s="274">
+      <c r="AK47" s="275">
         <v>22215</v>
       </c>
-      <c r="AL47" s="274">
+      <c r="AL47" s="275">
         <v>23960</v>
       </c>
-      <c r="AM47" s="274">
+      <c r="AM47" s="275">
         <v>22515</v>
       </c>
-      <c r="AN47" s="274">
+      <c r="AN47" s="275">
         <v>20719</v>
       </c>
-      <c r="AO47" s="274">
+      <c r="AO47" s="275">
         <v>19031</v>
       </c>
-      <c r="AP47" s="274">
+      <c r="AP47" s="275">
         <v>21295</v>
       </c>
-      <c r="AQ47" s="274">
+      <c r="AQ47" s="275">
         <v>23525</v>
       </c>
-      <c r="AR47" s="274">
+      <c r="AR47" s="275">
         <v>20195</v>
       </c>
-      <c r="AS47" s="274">
+      <c r="AS47" s="275">
         <v>24888</v>
       </c>
-      <c r="AT47" s="274">
+      <c r="AT47" s="275">
         <v>28896</v>
       </c>
-      <c r="AU47" s="274">
+      <c r="AU47" s="275">
         <v>15637</v>
       </c>
-      <c r="AV47" s="274">
+      <c r="AV47" s="275">
         <v>19983</v>
       </c>
-      <c r="AW47" s="274">
+      <c r="AW47" s="275">
         <v>21545</v>
       </c>
-      <c r="AX47" s="274">
+      <c r="AX47" s="275">
         <v>17673</v>
       </c>
-      <c r="AY47" s="274">
+      <c r="AY47" s="275">
         <v>19565</v>
       </c>
-      <c r="AZ47" s="277">
+      <c r="AZ47" s="278">
         <v>19146</v>
       </c>
-      <c r="BA47" s="276">
+      <c r="BA47" s="277">
         <v>17196</v>
       </c>
-      <c r="BB47" s="276">
+      <c r="BB47" s="277">
         <v>19835</v>
       </c>
-      <c r="BC47" s="276">
+      <c r="BC47" s="277">
         <v>22668</v>
       </c>
-      <c r="BD47" s="276">
+      <c r="BD47" s="277">
         <v>21855</v>
       </c>
-      <c r="BE47" s="276">
+      <c r="BE47" s="277">
         <v>24327</v>
       </c>
-      <c r="BF47" s="276">
+      <c r="BF47" s="277">
         <v>17958</v>
       </c>
-      <c r="BG47" s="276">
+      <c r="BG47" s="277">
         <v>18208</v>
       </c>
-      <c r="BH47" s="276">
+      <c r="BH47" s="277">
         <v>17880</v>
       </c>
-      <c r="BI47" s="276">
+      <c r="BI47" s="277">
         <v>20944</v>
       </c>
-      <c r="BJ47" s="276">
+      <c r="BJ47" s="277">
         <v>21100</v>
       </c>
-      <c r="BK47" s="276">
+      <c r="BK47" s="277">
         <v>20305</v>
       </c>
       <c r="BL47" s="77">
@@ -59906,7 +59914,7 @@
       </c>
     </row>
     <row r="48" spans="1:178" customFormat="1" ht="17">
-      <c r="A48" s="278"/>
+      <c r="A48" s="279"/>
       <c r="B48" s="265">
         <v>205337</v>
       </c>
@@ -59916,65 +59924,65 @@
       <c r="D48" s="72" t="s">
         <v>234</v>
       </c>
-      <c r="E48" s="274"/>
-      <c r="F48" s="274"/>
-      <c r="G48" s="274"/>
-      <c r="H48" s="274"/>
-      <c r="I48" s="274"/>
-      <c r="J48" s="274"/>
-      <c r="K48" s="274"/>
-      <c r="L48" s="274"/>
-      <c r="M48" s="274"/>
-      <c r="N48" s="274"/>
-      <c r="O48" s="274"/>
-      <c r="P48" s="274"/>
-      <c r="Q48" s="275"/>
-      <c r="R48" s="275"/>
-      <c r="S48" s="275"/>
-      <c r="T48" s="275"/>
-      <c r="U48" s="275"/>
-      <c r="V48" s="275"/>
-      <c r="W48" s="275"/>
-      <c r="X48" s="275"/>
-      <c r="Y48" s="275"/>
-      <c r="Z48" s="275"/>
-      <c r="AA48" s="275"/>
-      <c r="AB48" s="275"/>
-      <c r="AC48" s="274"/>
-      <c r="AD48" s="274"/>
-      <c r="AE48" s="274"/>
-      <c r="AF48" s="274"/>
-      <c r="AG48" s="274"/>
-      <c r="AH48" s="274"/>
-      <c r="AI48" s="274"/>
-      <c r="AJ48" s="274"/>
-      <c r="AK48" s="274"/>
-      <c r="AL48" s="274"/>
-      <c r="AM48" s="274"/>
-      <c r="AN48" s="274"/>
-      <c r="AO48" s="274"/>
-      <c r="AP48" s="274"/>
-      <c r="AQ48" s="274"/>
-      <c r="AR48" s="274"/>
-      <c r="AS48" s="274"/>
-      <c r="AT48" s="274"/>
-      <c r="AU48" s="274"/>
-      <c r="AV48" s="274"/>
-      <c r="AW48" s="274"/>
-      <c r="AX48" s="274"/>
-      <c r="AY48" s="274"/>
-      <c r="AZ48" s="277"/>
-      <c r="BA48" s="276"/>
-      <c r="BB48" s="276"/>
-      <c r="BC48" s="276"/>
-      <c r="BD48" s="276"/>
-      <c r="BE48" s="276"/>
-      <c r="BF48" s="276"/>
-      <c r="BG48" s="276"/>
-      <c r="BH48" s="276"/>
-      <c r="BI48" s="276"/>
-      <c r="BJ48" s="276"/>
-      <c r="BK48" s="276"/>
+      <c r="E48" s="275"/>
+      <c r="F48" s="275"/>
+      <c r="G48" s="275"/>
+      <c r="H48" s="275"/>
+      <c r="I48" s="275"/>
+      <c r="J48" s="275"/>
+      <c r="K48" s="275"/>
+      <c r="L48" s="275"/>
+      <c r="M48" s="275"/>
+      <c r="N48" s="275"/>
+      <c r="O48" s="275"/>
+      <c r="P48" s="275"/>
+      <c r="Q48" s="276"/>
+      <c r="R48" s="276"/>
+      <c r="S48" s="276"/>
+      <c r="T48" s="276"/>
+      <c r="U48" s="276"/>
+      <c r="V48" s="276"/>
+      <c r="W48" s="276"/>
+      <c r="X48" s="276"/>
+      <c r="Y48" s="276"/>
+      <c r="Z48" s="276"/>
+      <c r="AA48" s="276"/>
+      <c r="AB48" s="276"/>
+      <c r="AC48" s="275"/>
+      <c r="AD48" s="275"/>
+      <c r="AE48" s="275"/>
+      <c r="AF48" s="275"/>
+      <c r="AG48" s="275"/>
+      <c r="AH48" s="275"/>
+      <c r="AI48" s="275"/>
+      <c r="AJ48" s="275"/>
+      <c r="AK48" s="275"/>
+      <c r="AL48" s="275"/>
+      <c r="AM48" s="275"/>
+      <c r="AN48" s="275"/>
+      <c r="AO48" s="275"/>
+      <c r="AP48" s="275"/>
+      <c r="AQ48" s="275"/>
+      <c r="AR48" s="275"/>
+      <c r="AS48" s="275"/>
+      <c r="AT48" s="275"/>
+      <c r="AU48" s="275"/>
+      <c r="AV48" s="275"/>
+      <c r="AW48" s="275"/>
+      <c r="AX48" s="275"/>
+      <c r="AY48" s="275"/>
+      <c r="AZ48" s="278"/>
+      <c r="BA48" s="277"/>
+      <c r="BB48" s="277"/>
+      <c r="BC48" s="277"/>
+      <c r="BD48" s="277"/>
+      <c r="BE48" s="277"/>
+      <c r="BF48" s="277"/>
+      <c r="BG48" s="277"/>
+      <c r="BH48" s="277"/>
+      <c r="BI48" s="277"/>
+      <c r="BJ48" s="277"/>
+      <c r="BK48" s="277"/>
       <c r="BL48" s="233">
         <v>4656</v>
       </c>
@@ -60331,7 +60339,7 @@
       </c>
     </row>
     <row r="49" spans="1:178" customFormat="1" ht="34">
-      <c r="A49" s="278"/>
+      <c r="A49" s="279"/>
       <c r="B49" s="265">
         <v>229155</v>
       </c>
@@ -68191,6 +68199,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A29A70560454A24D9B372805159B7667" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="14f976c721eda7b2b215a20b4d5a78d8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bc76fe4c-a155-4cd4-b3ce-e749a30fe160" xmlns:ns3="be3055c3-5ee9-432b-9d2b-e9bb13d3524a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="403c36ed6babb1ecd579e11e58fd3547" ns2:_="" ns3:_="">
     <xsd:import namespace="bc76fe4c-a155-4cd4-b3ce-e749a30fe160"/>
@@ -68465,7 +68482,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Loretta xmlns="bc76fe4c-a155-4cd4-b3ce-e749a30fe160" xsi:nil="true"/>
@@ -68480,16 +68497,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4277783-1FC0-4518-9AC7-78441643C7FE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8ED3412-BBCC-49D1-9BBB-563663F97477}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -68508,7 +68524,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{771927D8-23AB-4166-821E-2FB8CF69E88F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -68517,12 +68533,4 @@
     <ds:schemaRef ds:uri="be3055c3-5ee9-432b-9d2b-e9bb13d3524a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4277783-1FC0-4518-9AC7-78441643C7FE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>